<commit_message>
put anything in BP in a notebook
</commit_message>
<xml_diff>
--- a/Data/BP.xlsx
+++ b/Data/BP.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pouniq/BloodPressure/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pouniq/BloodPressure/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{886287CF-1E49-344F-98F6-1265B2CE5172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{156EC06C-566F-0E4C-8602-E940CE6075A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="0" windowWidth="28040" windowHeight="17440" activeTab="1" xr2:uid="{ECD6C929-F296-5945-A84D-FAEE2E8C4A93}"/>
   </bookViews>
@@ -1432,6 +1432,12 @@
       <c r="E38">
         <v>121</v>
       </c>
+      <c r="F38">
+        <v>121</v>
+      </c>
+      <c r="G38">
+        <v>118</v>
+      </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="1"/>
@@ -1443,6 +1449,12 @@
       <c r="E39">
         <v>72</v>
       </c>
+      <c r="F39">
+        <v>66</v>
+      </c>
+      <c r="G39">
+        <v>75</v>
+      </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="1"/>
@@ -1454,6 +1466,12 @@
       <c r="E40">
         <v>60</v>
       </c>
+      <c r="F40">
+        <v>70</v>
+      </c>
+      <c r="G40">
+        <v>70</v>
+      </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="1"/>
@@ -1467,6 +1485,12 @@
       <c r="E41">
         <v>111</v>
       </c>
+      <c r="F41">
+        <v>132</v>
+      </c>
+      <c r="G41">
+        <v>127</v>
+      </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="1"/>
@@ -1478,6 +1502,12 @@
       <c r="E42">
         <v>73</v>
       </c>
+      <c r="F42">
+        <v>74</v>
+      </c>
+      <c r="G42">
+        <v>68</v>
+      </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" s="1"/>
@@ -1489,6 +1519,12 @@
       <c r="E43">
         <v>60</v>
       </c>
+      <c r="F43">
+        <v>73</v>
+      </c>
+      <c r="G43">
+        <v>60</v>
+      </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
@@ -1660,28 +1696,6 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="A26:A31"/>
-    <mergeCell ref="A32:A37"/>
-    <mergeCell ref="C35:C37"/>
-    <mergeCell ref="C50:C52"/>
-    <mergeCell ref="C53:C55"/>
-    <mergeCell ref="A2:A7"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="C5:C7"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="C20:C22"/>
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="A8:A13"/>
-    <mergeCell ref="A14:A19"/>
-    <mergeCell ref="A20:A25"/>
-    <mergeCell ref="A38:A43"/>
-    <mergeCell ref="A44:A49"/>
-    <mergeCell ref="A50:A55"/>
-    <mergeCell ref="B50:B55"/>
     <mergeCell ref="B56:B61"/>
     <mergeCell ref="A56:A61"/>
     <mergeCell ref="C56:C58"/>
@@ -1698,6 +1712,28 @@
     <mergeCell ref="C41:C43"/>
     <mergeCell ref="C44:C46"/>
     <mergeCell ref="C47:C49"/>
+    <mergeCell ref="A14:A19"/>
+    <mergeCell ref="A20:A25"/>
+    <mergeCell ref="A38:A43"/>
+    <mergeCell ref="A44:A49"/>
+    <mergeCell ref="A50:A55"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="A8:A13"/>
+    <mergeCell ref="A26:A31"/>
+    <mergeCell ref="A32:A37"/>
+    <mergeCell ref="C35:C37"/>
+    <mergeCell ref="C50:C52"/>
+    <mergeCell ref="C53:C55"/>
+    <mergeCell ref="B50:B55"/>
     <mergeCell ref="C29:C31"/>
     <mergeCell ref="C32:C34"/>
   </mergeCells>

</xml_diff>

<commit_message>
getting it working I Like what I am doing rn, need to know how to make that main class YKWIM, and I need to learn Polars It is fast
</commit_message>
<xml_diff>
--- a/Data/BP.xlsx
+++ b/Data/BP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pouniq/BloodPressure/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A0D29FFC-A735-1841-BD85-8CEB58677D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72E9FC1F-9701-2541-BED9-6C5C9E6D74DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="0" windowWidth="28040" windowHeight="17440" xr2:uid="{54DB268E-0F8D-AB4B-99D9-45144FAC5121}"/>
   </bookViews>
@@ -1594,15 +1594,42 @@
       <c r="D44" t="s">
         <v>9</v>
       </c>
+      <c r="E44">
+        <v>116</v>
+      </c>
+      <c r="F44">
+        <v>112</v>
+      </c>
+      <c r="G44">
+        <v>126</v>
+      </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D45" t="s">
         <v>10</v>
       </c>
+      <c r="E45">
+        <v>67</v>
+      </c>
+      <c r="F45">
+        <v>66</v>
+      </c>
+      <c r="G45">
+        <v>68</v>
+      </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D46" t="s">
         <v>11</v>
+      </c>
+      <c r="E46">
+        <v>56</v>
+      </c>
+      <c r="F46">
+        <v>78</v>
+      </c>
+      <c r="G46">
+        <v>72</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -1612,18 +1639,45 @@
       <c r="D47" t="s">
         <v>9</v>
       </c>
+      <c r="E47">
+        <v>123</v>
+      </c>
+      <c r="F47">
+        <v>129</v>
+      </c>
+      <c r="G47">
+        <v>133</v>
+      </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D48" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E48">
+        <v>86</v>
+      </c>
+      <c r="F48">
+        <v>65</v>
+      </c>
+      <c r="G48">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D49" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E49">
+        <v>60</v>
+      </c>
+      <c r="F49">
+        <v>71</v>
+      </c>
+      <c r="G49">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>9</v>
       </c>
@@ -1636,36 +1690,90 @@
       <c r="D50" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E50">
+        <v>127</v>
+      </c>
+      <c r="F50">
+        <v>137</v>
+      </c>
+      <c r="G50">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D51" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E51">
+        <v>75</v>
+      </c>
+      <c r="F51">
+        <v>72</v>
+      </c>
+      <c r="G51">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D52" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E52">
+        <v>67</v>
+      </c>
+      <c r="F52">
+        <v>85</v>
+      </c>
+      <c r="G52">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C53" t="s">
         <v>12</v>
       </c>
       <c r="D53" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E53">
+        <v>123</v>
+      </c>
+      <c r="F53">
+        <v>125</v>
+      </c>
+      <c r="G53">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D54" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E54">
+        <v>70</v>
+      </c>
+      <c r="F54">
+        <v>71</v>
+      </c>
+      <c r="G54">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D55" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E55">
+        <v>68</v>
+      </c>
+      <c r="F55">
+        <v>80</v>
+      </c>
+      <c r="G55">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>10</v>
       </c>
@@ -1679,17 +1787,17 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D57" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D58" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C59" t="s">
         <v>12</v>
       </c>
@@ -1697,12 +1805,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D60" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D61" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
done with EDA and Preprocessing and data file is complete
</commit_message>
<xml_diff>
--- a/Data/BP.xlsx
+++ b/Data/BP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pouniq/BloodPressure/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72E9FC1F-9701-2541-BED9-6C5C9E6D74DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{368095F5-3E34-514A-8AB8-4D4CACD329C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="0" windowWidth="28040" windowHeight="17440" xr2:uid="{54DB268E-0F8D-AB4B-99D9-45144FAC5121}"/>
   </bookViews>
@@ -1786,15 +1786,42 @@
       <c r="D56" t="s">
         <v>9</v>
       </c>
+      <c r="E56">
+        <v>132</v>
+      </c>
+      <c r="F56">
+        <v>114</v>
+      </c>
+      <c r="G56">
+        <v>116</v>
+      </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D57" t="s">
         <v>10</v>
       </c>
+      <c r="E57">
+        <v>68</v>
+      </c>
+      <c r="F57">
+        <v>59</v>
+      </c>
+      <c r="G57">
+        <v>72</v>
+      </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D58" t="s">
         <v>11</v>
+      </c>
+      <c r="E58">
+        <v>64</v>
+      </c>
+      <c r="F58">
+        <v>68</v>
+      </c>
+      <c r="G58">
+        <v>66</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -1804,15 +1831,42 @@
       <c r="D59" t="s">
         <v>9</v>
       </c>
+      <c r="E59">
+        <v>133</v>
+      </c>
+      <c r="F59">
+        <v>122</v>
+      </c>
+      <c r="G59">
+        <v>123</v>
+      </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D60" t="s">
         <v>10</v>
       </c>
+      <c r="E60">
+        <v>73</v>
+      </c>
+      <c r="F60">
+        <v>63</v>
+      </c>
+      <c r="G60">
+        <v>70</v>
+      </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D61" t="s">
         <v>11</v>
+      </c>
+      <c r="E61">
+        <v>66</v>
+      </c>
+      <c r="F61">
+        <v>68</v>
+      </c>
+      <c r="G61">
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>